<commit_message>
update Bom and schematic image from most current changes
changed r9 resistor value to 10k. Routed the PG pin from tps61232 to pico pin 20, co-opting 100k resistor r3 as a pullup to 3v3 rail
</commit_message>
<xml_diff>
--- a/Datasheets/BOM_Prototype_Prototype camera board_2026-10-25.xlsx
+++ b/Datasheets/BOM_Prototype_Prototype camera board_2026-10-25.xlsx
@@ -313,7 +313,7 @@
     <t>10kΩ</t>
   </si>
   <si>
-    <t>R1,R2,R4</t>
+    <t>R1,R2,R4,R9</t>
   </si>
   <si>
     <t>R0805</t>
@@ -334,7 +334,7 @@
     <t>100kΩ</t>
   </si>
   <si>
-    <t>R3,R9</t>
+    <t>R3</t>
   </si>
   <si>
     <t>0805W8F1003T5E</t>
@@ -1371,7 +1371,7 @@
         <v>98</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="s">
         <v>99</v>
@@ -1403,7 +1403,7 @@
         <v>105</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" t="s">
         <v>106</v>

</xml_diff>